<commit_message>
Force EUR as currency; filter sold funds;  add sell dates; fomat x-axis
</commit_message>
<xml_diff>
--- a/_Codex/Data/Input_Data/fund_manual_values.xlsx
+++ b/_Codex/Data/Input_Data/fund_manual_values.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="612" yWindow="516" windowWidth="21852" windowHeight="10260"/>
+    <workbookView xWindow="615" yWindow="510" windowWidth="21855" windowHeight="10260" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="ScalarValues" sheetId="1" r:id="rId1"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="468" uniqueCount="204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="478" uniqueCount="209">
   <si>
     <t>isin</t>
   </si>
@@ -628,16 +628,36 @@
   </si>
   <si>
     <t>DKB</t>
+  </si>
+  <si>
+    <t>ISHSV-MSCI ACWI DL A</t>
+  </si>
+  <si>
+    <t>IE00B6R52259</t>
+  </si>
+  <si>
+    <t>2026-05-27</t>
+  </si>
+  <si>
+    <t>manual</t>
+  </si>
+  <si>
+    <t>2024-05-27</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -660,8 +680,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -963,8 +986,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G12"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
+  <dimension ref="A1:G13"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="54.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.42578125" style="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" t="s">
@@ -973,7 +1000,7 @@
       <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D1" t="s">
@@ -996,7 +1023,7 @@
       <c r="B2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="1" t="s">
         <v>8</v>
       </c>
       <c r="D2" t="s">
@@ -1019,7 +1046,7 @@
       <c r="B3" t="s">
         <v>13</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D3" t="s">
@@ -1042,7 +1069,7 @@
       <c r="B4" t="s">
         <v>17</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="1" t="s">
         <v>18</v>
       </c>
       <c r="D4" t="s">
@@ -1065,7 +1092,7 @@
       <c r="B5" t="s">
         <v>23</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="1" t="s">
         <v>24</v>
       </c>
       <c r="D5" t="s">
@@ -1088,7 +1115,7 @@
       <c r="B6" t="s">
         <v>27</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="1" t="s">
         <v>28</v>
       </c>
       <c r="D6" t="s">
@@ -1111,7 +1138,7 @@
       <c r="B7" t="s">
         <v>31</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="1" t="s">
         <v>32</v>
       </c>
       <c r="D7" t="s">
@@ -1134,7 +1161,7 @@
       <c r="B8" t="s">
         <v>36</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="1" t="s">
         <v>37</v>
       </c>
       <c r="D8" t="s">
@@ -1157,7 +1184,7 @@
       <c r="B9" t="s">
         <v>40</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="1" t="s">
         <v>41</v>
       </c>
       <c r="D9" t="s">
@@ -1180,7 +1207,7 @@
       <c r="B10" t="s">
         <v>44</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="1" t="s">
         <v>45</v>
       </c>
       <c r="D10" t="s">
@@ -1203,7 +1230,7 @@
       <c r="B11" t="s">
         <v>49</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="1" t="s">
         <v>50</v>
       </c>
       <c r="D11" t="s">
@@ -1226,7 +1253,7 @@
       <c r="B12" t="s">
         <v>53</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="1" t="s">
         <v>54</v>
       </c>
       <c r="D12" t="s">
@@ -1242,15 +1269,39 @@
         <v>55</v>
       </c>
     </row>
+    <row r="13" spans="1:7">
+      <c r="A13" t="s">
+        <v>205</v>
+      </c>
+      <c r="B13" t="s">
+        <v>204</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="D13" t="s">
+        <v>9</v>
+      </c>
+      <c r="E13" t="s">
+        <v>10</v>
+      </c>
+      <c r="F13" t="s">
+        <v>203</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>207</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E56"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
@@ -2211,14 +2262,17 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D26"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
+  <dimension ref="A1:D27"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="11.42578125" style="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>57</v>
       </c>
       <c r="C1" t="s">
@@ -2232,7 +2286,7 @@
       <c r="A2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="1" t="s">
         <v>8</v>
       </c>
       <c r="C2" t="s">
@@ -2246,7 +2300,7 @@
       <c r="A3" t="s">
         <v>6</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="1" t="s">
         <v>62</v>
       </c>
       <c r="C3" t="s">
@@ -2260,7 +2314,7 @@
       <c r="A4" t="s">
         <v>12</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="1" t="s">
         <v>14</v>
       </c>
       <c r="C4" t="s">
@@ -2274,7 +2328,7 @@
       <c r="A5" t="s">
         <v>12</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="1" t="s">
         <v>73</v>
       </c>
       <c r="C5" t="s">
@@ -2288,7 +2342,7 @@
       <c r="A6" t="s">
         <v>16</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="1" t="s">
         <v>18</v>
       </c>
       <c r="C6" t="s">
@@ -2302,7 +2356,7 @@
       <c r="A7" t="s">
         <v>16</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="1" t="s">
         <v>82</v>
       </c>
       <c r="C7" t="s">
@@ -2316,7 +2370,7 @@
       <c r="A8" t="s">
         <v>16</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C8" t="s">
@@ -2330,7 +2384,7 @@
       <c r="A9" t="s">
         <v>22</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="1" t="s">
         <v>24</v>
       </c>
       <c r="C9" t="s">
@@ -2344,7 +2398,7 @@
       <c r="A10" t="s">
         <v>22</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="1" t="s">
         <v>90</v>
       </c>
       <c r="C10" t="s">
@@ -2358,7 +2412,7 @@
       <c r="A11" t="s">
         <v>26</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="1" t="s">
         <v>28</v>
       </c>
       <c r="C11" t="s">
@@ -2372,7 +2426,7 @@
       <c r="A12" t="s">
         <v>26</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="1" t="s">
         <v>98</v>
       </c>
       <c r="C12" t="s">
@@ -2386,7 +2440,7 @@
       <c r="A13" t="s">
         <v>30</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="1" t="s">
         <v>32</v>
       </c>
       <c r="C13" t="s">
@@ -2400,7 +2454,7 @@
       <c r="A14" t="s">
         <v>30</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="1" t="s">
         <v>105</v>
       </c>
       <c r="C14" t="s">
@@ -2414,7 +2468,7 @@
       <c r="A15" t="s">
         <v>30</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="1" t="s">
         <v>33</v>
       </c>
       <c r="C15" t="s">
@@ -2428,7 +2482,7 @@
       <c r="A16" t="s">
         <v>35</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="1" t="s">
         <v>37</v>
       </c>
       <c r="C16" t="s">
@@ -2442,7 +2496,7 @@
       <c r="A17" t="s">
         <v>35</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="1" t="s">
         <v>112</v>
       </c>
       <c r="C17" t="s">
@@ -2456,7 +2510,7 @@
       <c r="A18" t="s">
         <v>39</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="1" t="s">
         <v>41</v>
       </c>
       <c r="C18" t="s">
@@ -2470,7 +2524,7 @@
       <c r="A19" t="s">
         <v>39</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="1" t="s">
         <v>119</v>
       </c>
       <c r="C19" t="s">
@@ -2484,7 +2538,7 @@
       <c r="A20" t="s">
         <v>43</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="1" t="s">
         <v>45</v>
       </c>
       <c r="C20" t="s">
@@ -2498,7 +2552,7 @@
       <c r="A21" t="s">
         <v>43</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="1" t="s">
         <v>126</v>
       </c>
       <c r="C21" t="s">
@@ -2512,7 +2566,7 @@
       <c r="A22" t="s">
         <v>43</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B22" s="1" t="s">
         <v>46</v>
       </c>
       <c r="C22" t="s">
@@ -2526,7 +2580,7 @@
       <c r="A23" t="s">
         <v>48</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B23" s="1" t="s">
         <v>50</v>
       </c>
       <c r="C23" t="s">
@@ -2540,7 +2594,7 @@
       <c r="A24" t="s">
         <v>48</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B24" s="1" t="s">
         <v>133</v>
       </c>
       <c r="C24" t="s">
@@ -2554,7 +2608,7 @@
       <c r="A25" t="s">
         <v>52</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B25" s="1" t="s">
         <v>54</v>
       </c>
       <c r="C25" t="s">
@@ -2568,7 +2622,7 @@
       <c r="A26" t="s">
         <v>52</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B26" s="1" t="s">
         <v>140</v>
       </c>
       <c r="C26" t="s">
@@ -2576,6 +2630,20 @@
       </c>
       <c r="D26" t="s">
         <v>200</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4">
+      <c r="A27" t="s">
+        <v>205</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="C27">
+        <v>2</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>207</v>
       </c>
     </row>
   </sheetData>

</xml_diff>